<commit_message>
OK200-68 updated responsive styling, updates login, 403, verified logging in/out of users
</commit_message>
<xml_diff>
--- a/translations.xlsx
+++ b/translations.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,10 +449,10 @@
         <v>shared.header.bookCatalog</v>
       </c>
       <c r="B5" t="str">
-        <v>Book Catalog</v>
+        <v>Books Catalog</v>
       </c>
       <c r="C5" t="str">
-        <v>Book Catalog</v>
+        <v>Books Catalog</v>
       </c>
     </row>
     <row r="6">
@@ -621,13 +621,63 @@
       </c>
     </row>
     <row r="21">
+      <c r="A21" t="str">
+        <v>shared.header.userMenu</v>
+      </c>
       <c r="B21" t="str">
-        <v/>
+        <v>User Menu</v>
+      </c>
+      <c r="C21" t="str">
+        <v>User Menu</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>shared.header.navigation</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Navigation</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Navigation</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>shared.header.openNav</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Open Navigation</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Open Navigation</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>shared.header.libSystem</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Library System</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Library System</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>shared.header.mngmtPortal</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Management Portal</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Management Portal</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C25"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>